<commit_message>
update for 4 A,B,C
</commit_message>
<xml_diff>
--- a/week-01/GTrends_milkshake_hamburger_2024.csv/Ex4C_GTrends.xlsx
+++ b/week-01/GTrends_milkshake_hamburger_2024.csv/Ex4C_GTrends.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sthef\data-analytics\week-01\GTrends_milkshake_hamburger_2024.csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{641B35C9-A80A-48A9-972C-4B3721968DF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC05EB20-DD08-4A9B-9A26-E54B211F977B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1020" yWindow="1824" windowWidth="17040" windowHeight="8916" xr2:uid="{FFC9F9BE-BA05-4A56-BC1B-0ECC51FCB96D}"/>
+    <workbookView xWindow="2856" yWindow="2268" windowWidth="17040" windowHeight="8916" xr2:uid="{FFC9F9BE-BA05-4A56-BC1B-0ECC51FCB96D}"/>
   </bookViews>
   <sheets>
     <sheet name="By search term" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="61">
   <si>
     <t>Carolina del Sur</t>
   </si>
@@ -214,6 +214,12 @@
   </si>
   <si>
     <t xml:space="preserve"> 1/2/24 - 28/2/25</t>
+  </si>
+  <si>
+    <t>Nuevo Mexico</t>
+  </si>
+  <si>
+    <t>Michigan</t>
   </si>
 </sst>
 </file>
@@ -1559,7 +1565,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="C25" s="2">
         <v>0.67</v>
@@ -1780,7 +1786,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="C38" s="2">
         <v>0.67</v>

</xml_diff>